<commit_message>
Correct NIL mechanism in BC model: third-party (uncapped), not routed through school cap
The roster/NIL is contracted directly by the SPV as a third party — uncapped and
stacked ON TOP of the school's ~$3M men's-basketball slice of the House cap, not
routed through it. Real constraint is the NIL Go FMV/valid-business-purpose
clearinghouse, which the docuseries-backed model is structured to pass. Relabeled
the roster line and added an NIL-structure section to the Read me.
</commit_message>
<xml_diff>
--- a/cinderella/Outputs/2026-07-23-bc-full-stack-model.xlsx
+++ b/cinderella/Outputs/2026-07-23-bc-full-stack-model.xlsx
@@ -615,7 +615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -707,67 +707,119 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>The two headline answers</t>
+          <t>NIL structure (important)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>• $30M+ SPV: reached by the SHOW layer, not the gym. Bucket 1 alone caps ~$11-19M to the SPV.</t>
+          <t>• Roster/NIL is THIRD-PARTY: the SPV contracts players directly (like a collective). It is UNCAPPED and is NOT</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>• Duke-level ($44.8M): not TEAM revenue in 5 yrs, but ENTERPRISE total is Duke-adjacent (base) to Duke-level (reach)</t>
+          <t xml:space="preserve">   routed through the school's House rev-share cap. The school's cap (~$20.5M; ~$3M to men's basketball after football)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">   because Duke monetizes zero media layer. Team-medium + media-heavy = Duke total, different engine.</t>
+          <t xml:space="preserve">   stays with the school and STACKS on top of our ~$12M -&gt; ~$15M total player comp, ACC-competitive.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr"/>
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>• The real constraint is NIL Go (Deloitte clearinghouse): any 3rd-party deal &gt;=$600 must clear a 'fair market value' +</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Key risk</t>
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   'valid business purpose' test. Cinderella passes cleanly because the NIL is backed by real commerce (docuseries</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">   appearances, sponsor activations, merch, likeness) — where a pure booster collective paying 'to retain' fails.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>The two headline answers</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>• $30M+ SPV: reached by the SHOW layer, not the gym. Bucket 1 alone caps ~$11-19M to the SPV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>• Duke-level ($44.8M): not TEAM revenue in 5 yrs, but ENTERPRISE total is Duke-adjacent (base) to Duke-level (reach)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   because Duke monetizes zero media layer. Team-medium + media-heavy = Duke total, different engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Key risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
           <t>• The delta between Base and Reach is almost entirely Bucket 2 — i.e., does the documentary land nationally?</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">  The roster still costs $12-13M regardless. That is the bet.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>Sources: EADA (BC $8.33M rev / $8.67M exp; Duke $44.8M); ACC ~$45M/school -&gt; $35-65M merit band; Van Wagner MMR; Conte 8,606.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>NOT financial advice — a planning model with estimated inputs. Verify all figures before external use.</t>
         </is>
@@ -1168,10 +1220,14 @@
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t>Roster / NIL (House cap + collective)</t>
-        </is>
-      </c>
-      <c r="B27" s="12" t="inlineStr"/>
+          <t>Roster / NIL (third-party, via SPV)</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>uncapped; ON TOP of school's ~$3M cap; NIL Go FMV-vetted</t>
+        </is>
+      </c>
       <c r="C27" s="13" t="n">
         <v>12</v>
       </c>
@@ -1632,7 +1688,7 @@
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>House cap + collective</t>
+          <t>3rd-party NIL, uncapped; on top of school cap</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add NCAA units distribution reference note + unit-retention toggle in BC model
- Process note: per-conference NCAA units distribution (equal vs earned), confidence
  flags, A-10 75/25 discrepancy flag, site-selection implication
- BC model: new 'NCAA Tournament Units' assumptions block (units earned, unit value,
  conference unit-retention % toggle) + contingent tournament-run upside section in the
  P&L (retained units -> SPV 80%), kept separate from the Layer 3 conference fee to
  avoid double-count; Read me updated
</commit_message>
<xml_diff>
--- a/cinderella/Outputs/2026-07-23-bc-full-stack-model.xlsx
+++ b/cinderella/Outputs/2026-07-23-bc-full-stack-model.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
     <numFmt numFmtId="165" formatCode="0.00&quot;x&quot;"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -76,6 +76,11 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001F3352"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001E5631"/>
       <sz val="11"/>
     </font>
     <font>
@@ -161,14 +166,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -178,6 +180,9 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -241,10 +246,16 @@
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="9" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -615,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A32"/>
+  <dimension ref="A1:A38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -788,38 +799,76 @@
       <c r="A26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>Key risk</t>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>NCAA tournament units (contingent upside)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>• The delta between Base and Reach is almost entirely Bucket 2 — i.e., does the documentary land nationally?</t>
+          <t>• A run earns 'units' the conference distributes. Whether the SCHOOL keeps them depends on conference policy:</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">   A-10 keeps ~75%, WCC uneven, Big Ten/SEC ~pooled (school keeps little), ACC transitioning. Toggle the</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   'Conference unit-retention %' input per school. Retained units are revenue above baseline -&gt; SPV takes 80%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>• Shown as CONTINGENT upside (a run isn't guaranteed) and kept SEPARATE from the Layer 3 conference fee to avoid double-count.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Key risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>• The delta between Base and Reach is almost entirely Bucket 2 — i.e., does the documentary land nationally?</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">  The roster still costs $12-13M regardless. That is the bet.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>Sources: EADA (BC $8.33M rev / $8.67M exp; Duke $44.8M); ACC ~$45M/school -&gt; $35-65M merit band; Van Wagner MMR; Conte 8,606.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>NOT financial advice — a planning model with estimated inputs. Verify all figures before external use.</t>
         </is>
@@ -836,7 +885,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1210,7 +1259,7 @@
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>SPV COSTS</t>
+          <t>NCAA TOURNAMENT UNITS (contingent upside)</t>
         </is>
       </c>
       <c r="B26" s="10" t="n"/>
@@ -1220,95 +1269,107 @@
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t>Roster / NIL (third-party, via SPV)</t>
+          <t>Units earned in a run (6-yr)</t>
         </is>
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>uncapped; ON TOP of school's ~$3M cap; NIL Go FMV-vetted</t>
+          <t>count of units from a tourney run</t>
         </is>
       </c>
       <c r="C27" s="13" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="D27" s="13" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>SPV operating costs</t>
+          <t>Unit value ($M, 6-yr total)</t>
         </is>
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>ops / staff / on-site</t>
+          <t>~$2M each over 6 yrs</t>
         </is>
       </c>
       <c r="C28" s="13" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="D28" s="13" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="inlineStr">
-        <is>
-          <t>PARENT / STRUCTURE</t>
-        </is>
-      </c>
-      <c r="B29" s="10" t="n"/>
-      <c r="C29" s="10" t="n"/>
-      <c r="D29" s="10" t="n"/>
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>Conference unit-retention %</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>TOGGLE per school: A10=75%, WCC uneven, B1G/SEC~0 (pooled), ACC transitioning</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D29" s="14" t="n">
+        <v>0.75</v>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="inlineStr">
-        <is>
-          <t>Parent equity in SPV</t>
-        </is>
-      </c>
-      <c r="B30" s="12" t="inlineStr"/>
-      <c r="C30" s="14" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="D30" s="14" t="n">
-        <v>0.4</v>
-      </c>
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>SPV COSTS</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="n"/>
+      <c r="C30" s="10" t="n"/>
+      <c r="D30" s="10" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>Management fee (% of SPV revenue)</t>
-        </is>
-      </c>
-      <c r="B31" s="12" t="inlineStr"/>
-      <c r="C31" s="14" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="D31" s="14" t="n">
-        <v>0.02</v>
+          <t>Roster / NIL (third-party, via SPV)</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>uncapped; ON TOP of school's ~$3M cap; NIL Go FMV-vetted</t>
+        </is>
+      </c>
+      <c r="C31" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="D31" s="13" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>Franchise fee (one-time)</t>
-        </is>
-      </c>
-      <c r="B32" s="12" t="inlineStr"/>
+          <t>SPV operating costs</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>ops / staff / on-site</t>
+        </is>
+      </c>
       <c r="C32" s="13" t="n">
         <v>1.5</v>
       </c>
       <c r="D32" s="13" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="10" t="inlineStr">
         <is>
-          <t>SEED WATERFALL (parent-level)</t>
+          <t>PARENT / STRUCTURE</t>
         </is>
       </c>
       <c r="B33" s="10" t="n"/>
@@ -1318,72 +1379,124 @@
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>Seed raised</t>
-        </is>
-      </c>
-      <c r="B34" s="12" t="inlineStr">
-        <is>
-          <t>Ankur / Tabor</t>
-        </is>
-      </c>
-      <c r="C34" s="13" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="D34" s="13" t="n">
-        <v>1.5</v>
+          <t>Parent equity in SPV</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="inlineStr"/>
+      <c r="C34" s="14" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D34" s="14" t="n">
+        <v>0.4</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="11" t="inlineStr">
         <is>
-          <t>Tier 1 rate — to 1x</t>
-        </is>
-      </c>
-      <c r="B35" s="12" t="inlineStr">
-        <is>
-          <t>of gross</t>
-        </is>
-      </c>
+          <t>Management fee (% of SPV revenue)</t>
+        </is>
+      </c>
+      <c r="B35" s="12" t="inlineStr"/>
       <c r="C35" s="14" t="n">
-        <v>0.5</v>
+        <v>0.02</v>
       </c>
       <c r="D35" s="14" t="n">
-        <v>0.5</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
         <is>
+          <t>Franchise fee (one-time)</t>
+        </is>
+      </c>
+      <c r="B36" s="12" t="inlineStr"/>
+      <c r="C36" s="13" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D36" s="13" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>SEED WATERFALL (parent-level)</t>
+        </is>
+      </c>
+      <c r="B37" s="10" t="n"/>
+      <c r="C37" s="10" t="n"/>
+      <c r="D37" s="10" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>Seed raised</t>
+        </is>
+      </c>
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>Ankur / Tabor</t>
+        </is>
+      </c>
+      <c r="C38" s="13" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D38" s="13" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="11" t="inlineStr">
+        <is>
+          <t>Tier 1 rate — to 1x</t>
+        </is>
+      </c>
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>of gross</t>
+        </is>
+      </c>
+      <c r="C39" s="14" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D39" s="14" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="11" t="inlineStr">
+        <is>
           <t>Tier 2 rate — 1x to 2x</t>
         </is>
       </c>
-      <c r="B36" s="12" t="inlineStr">
+      <c r="B40" s="12" t="inlineStr">
         <is>
           <t>of gross</t>
         </is>
       </c>
-      <c r="C36" s="14" t="n">
+      <c r="C40" s="14" t="n">
         <v>0.1</v>
       </c>
-      <c r="D36" s="14" t="n">
+      <c r="D40" s="14" t="n">
         <v>0.1</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="11" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="11" t="inlineStr">
         <is>
           <t>Tier 3 rate — after 2x</t>
         </is>
       </c>
-      <c r="B37" s="12" t="inlineStr">
+      <c r="B41" s="12" t="inlineStr">
         <is>
           <t>of gross</t>
         </is>
       </c>
-      <c r="C37" s="14" t="n">
+      <c r="C41" s="14" t="n">
         <v>0.15</v>
       </c>
-      <c r="D37" s="14" t="n">
+      <c r="D41" s="14" t="n">
         <v>0.15</v>
       </c>
     </row>
@@ -1398,7 +1511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1679,11 +1792,11 @@
         </is>
       </c>
       <c r="B19" s="17">
-        <f>-Assumptions!C27</f>
+        <f>-Assumptions!C31</f>
         <v/>
       </c>
       <c r="C19" s="17">
-        <f>-Assumptions!D27</f>
+        <f>-Assumptions!D31</f>
         <v/>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -1699,11 +1812,11 @@
         </is>
       </c>
       <c r="B20" s="17">
-        <f>-Assumptions!C28</f>
+        <f>-Assumptions!C32</f>
         <v/>
       </c>
       <c r="C20" s="17">
-        <f>-Assumptions!D28</f>
+        <f>-Assumptions!D32</f>
         <v/>
       </c>
       <c r="D20" s="12" t="inlineStr"/>
@@ -1715,11 +1828,11 @@
         </is>
       </c>
       <c r="B21" s="17">
-        <f>-Assumptions!C31*B17</f>
+        <f>-Assumptions!C35*B17</f>
         <v/>
       </c>
       <c r="C21" s="17">
-        <f>-Assumptions!D31*C17</f>
+        <f>-Assumptions!D35*C17</f>
         <v/>
       </c>
       <c r="D21" s="12" t="inlineStr">
@@ -1781,11 +1894,11 @@
         </is>
       </c>
       <c r="B25" s="17">
-        <f>B24*Assumptions!C30</f>
+        <f>B24*Assumptions!C34</f>
         <v/>
       </c>
       <c r="C25" s="17">
-        <f>C24*Assumptions!D30</f>
+        <f>C24*Assumptions!D34</f>
         <v/>
       </c>
       <c r="D25" s="12" t="inlineStr"/>
@@ -1797,11 +1910,11 @@
         </is>
       </c>
       <c r="B26" s="17">
-        <f>B24*(1-Assumptions!C30)</f>
+        <f>B24*(1-Assumptions!C34)</f>
         <v/>
       </c>
       <c r="C26" s="17">
-        <f>C24*(1-Assumptions!D30)</f>
+        <f>C24*(1-Assumptions!D34)</f>
         <v/>
       </c>
       <c r="D26" s="12" t="inlineStr"/>
@@ -1813,11 +1926,11 @@
         </is>
       </c>
       <c r="B27" s="24">
-        <f>B25+Assumptions!C31*B17+Assumptions!C32</f>
+        <f>B25+Assumptions!C35*B17+Assumptions!C36</f>
         <v/>
       </c>
       <c r="C27" s="24">
-        <f>C25+Assumptions!D31*C17+Assumptions!D32</f>
+        <f>C25+Assumptions!D35*C17+Assumptions!D36</f>
         <v/>
       </c>
       <c r="D27" s="25" t="inlineStr">
@@ -1879,7 +1992,7 @@
     <row r="31">
       <c r="A31" s="10" t="inlineStr">
         <is>
-          <t>BENCHMARK</t>
+          <t>TOURNAMENT-RUN UPSIDE (contingent — NOT in base SPV revenue above)</t>
         </is>
       </c>
       <c r="B31" s="10" t="n"/>
@@ -1887,58 +2000,128 @@
       <c r="D31" s="10" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="11" t="inlineStr">
+      <c r="A32" s="15" t="inlineStr">
+        <is>
+          <t>Retained NCAA unit revenue (6-yr total)</t>
+        </is>
+      </c>
+      <c r="B32" s="16">
+        <f>Assumptions!C27*Assumptions!C28*Assumptions!C29</f>
+        <v/>
+      </c>
+      <c r="C32" s="16">
+        <f>Assumptions!D27*Assumptions!D28*Assumptions!D29</f>
+        <v/>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>units x value x retention %</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="27" t="inlineStr">
+        <is>
+          <t>SPV share of retained units (80%)</t>
+        </is>
+      </c>
+      <c r="B33" s="28">
+        <f>B32*Assumptions!C7</f>
+        <v/>
+      </c>
+      <c r="C33" s="28">
+        <f>C32*Assumptions!D7</f>
+        <v/>
+      </c>
+      <c r="D33" s="20" t="inlineStr">
+        <is>
+          <t>units are revenue above baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  annualized SPV share (÷6 yrs)</t>
+        </is>
+      </c>
+      <c r="B34" s="17">
+        <f>B33/6</f>
+        <v/>
+      </c>
+      <c r="C34" s="17">
+        <f>C33/6</f>
+        <v/>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>separate from Layer 3 conf. fee — avoid double-count</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t>BENCHMARK</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="n"/>
+      <c r="C35" s="10" t="n"/>
+      <c r="D35" s="10" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
         <is>
           <t>Duke men's basketball revenue (2023-24)</t>
         </is>
       </c>
-      <c r="B32" s="17" t="n">
+      <c r="B36" s="17" t="n">
         <v>44.8</v>
       </c>
-      <c r="C32" s="17" t="n">
+      <c r="C36" s="17" t="n">
         <v>44.8</v>
       </c>
-      <c r="D32" s="12" t="inlineStr">
+      <c r="D36" s="12" t="inlineStr">
         <is>
           <t>EADA #1 in nation</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="15" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="15" t="inlineStr">
         <is>
           <t>Cinderella-BC enterprise total (team+show)</t>
         </is>
       </c>
-      <c r="B33" s="16">
+      <c r="B37" s="16">
         <f>B6+B11+B12+B15</f>
         <v/>
       </c>
-      <c r="C33" s="16">
+      <c r="C37" s="16">
         <f>C6+C11+C12+C15</f>
         <v/>
       </c>
-      <c r="D33" s="12" t="inlineStr">
+      <c r="D37" s="12" t="inlineStr">
         <is>
           <t>all revenue the venture touches</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="23" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="23" t="inlineStr">
         <is>
           <t>% of Duke (enterprise basis)</t>
         </is>
       </c>
-      <c r="B34" s="27">
-        <f>B33/B32</f>
-        <v/>
-      </c>
-      <c r="C34" s="27">
-        <f>C33/C32</f>
-        <v/>
-      </c>
-      <c r="D34" s="25" t="inlineStr">
+      <c r="B38" s="29">
+        <f>B37/B36</f>
+        <v/>
+      </c>
+      <c r="C38" s="29">
+        <f>C37/C36</f>
+        <v/>
+      </c>
+      <c r="D38" s="25" t="inlineStr">
         <is>
           <t>team-medium + media-heavy = Duke total</t>
         </is>
@@ -1979,7 +2162,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="28" t="inlineStr">
+      <c r="A3" s="30" t="inlineStr">
         <is>
           <t>Note: real waterfall is CUMULATIVE across all SPVs &amp; years — see capital-deployment workbook. This shows one BC season as if first money in.</t>
         </is>
@@ -2034,11 +2217,11 @@
         </is>
       </c>
       <c r="B7" s="17">
-        <f>(Assumptions!C34/Assumptions!C35)</f>
+        <f>(Assumptions!C38/Assumptions!C39)</f>
         <v/>
       </c>
       <c r="C7" s="17">
-        <f>(Assumptions!D34/Assumptions!D35)</f>
+        <f>(Assumptions!D38/Assumptions!D39)</f>
         <v/>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -2054,11 +2237,11 @@
         </is>
       </c>
       <c r="B8" s="17">
-        <f>(Assumptions!C34/Assumptions!C35+Assumptions!C34/Assumptions!C36)</f>
+        <f>(Assumptions!C38/Assumptions!C39+Assumptions!C38/Assumptions!C40)</f>
         <v/>
       </c>
       <c r="C8" s="17">
-        <f>(Assumptions!D34/Assumptions!D35+Assumptions!D34/Assumptions!D36)</f>
+        <f>(Assumptions!D38/Assumptions!D39+Assumptions!D38/Assumptions!D40)</f>
         <v/>
       </c>
       <c r="D8" s="12" t="inlineStr">
@@ -2074,11 +2257,11 @@
         </is>
       </c>
       <c r="B9" s="19">
-        <f>Assumptions!C35*MIN(B6,(Assumptions!C34/Assumptions!C35))+Assumptions!C36*MIN(MAX(B6-(Assumptions!C34/Assumptions!C35),0),Assumptions!C34/Assumptions!C36)+Assumptions!C37*MAX(B6-(Assumptions!C34/Assumptions!C35+Assumptions!C34/Assumptions!C36),0)</f>
+        <f>Assumptions!C39*MIN(B6,(Assumptions!C38/Assumptions!C39))+Assumptions!C40*MIN(MAX(B6-(Assumptions!C38/Assumptions!C39),0),Assumptions!C38/Assumptions!C40)+Assumptions!C41*MAX(B6-(Assumptions!C38/Assumptions!C39+Assumptions!C38/Assumptions!C40),0)</f>
         <v/>
       </c>
       <c r="C9" s="19">
-        <f>Assumptions!D35*MIN(C6,(Assumptions!D34/Assumptions!D35))+Assumptions!D36*MIN(MAX(C6-(Assumptions!D34/Assumptions!D35),0),Assumptions!D34/Assumptions!D36)+Assumptions!D37*MAX(C6-(Assumptions!D34/Assumptions!D35+Assumptions!D34/Assumptions!D36),0)</f>
+        <f>Assumptions!D39*MIN(C6,(Assumptions!D38/Assumptions!D39))+Assumptions!D40*MIN(MAX(C6-(Assumptions!D38/Assumptions!D39),0),Assumptions!D38/Assumptions!D40)+Assumptions!D41*MAX(C6-(Assumptions!D38/Assumptions!D39+Assumptions!D38/Assumptions!D40),0)</f>
         <v/>
       </c>
       <c r="D9" s="20" t="inlineStr">
@@ -2093,12 +2276,12 @@
           <t>Seed cumulative MOIC (this period)</t>
         </is>
       </c>
-      <c r="B10" s="29">
-        <f>B9/Assumptions!C34</f>
-        <v/>
-      </c>
-      <c r="C10" s="29">
-        <f>C9/Assumptions!D34</f>
+      <c r="B10" s="31">
+        <f>B9/Assumptions!C38</f>
+        <v/>
+      </c>
+      <c r="C10" s="31">
+        <f>C9/Assumptions!D38</f>
         <v/>
       </c>
       <c r="D10" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Correct A-10 units retention to 100% (St. Joe's AD, primary source)
Supersedes the older public 75/25 figure. Updated the units reference note and the
BC model's retention-toggle reference strings; A-10 flagged as the best unit-capture
conference for the SPV thesis.
</commit_message>
<xml_diff>
--- a/cinderella/Outputs/2026-07-23-bc-full-stack-model.xlsx
+++ b/cinderella/Outputs/2026-07-23-bc-full-stack-model.xlsx
@@ -815,7 +815,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">   A-10 keeps ~75%, WCC uneven, Big Ten/SEC ~pooled (school keeps little), ACC transitioning. Toggle the</t>
+          <t xml:space="preserve">   A-10 keeps 100% (St. Joe's AD), WCC uneven, Big Ten/SEC ~pooled (school keeps little), ACC transitioning. Toggle the</t>
         </is>
       </c>
     </row>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>TOGGLE per school: A10=75%, WCC uneven, B1G/SEC~0 (pooled), ACC transitioning</t>
+          <t>TOGGLE per school: A10=100% (St.Joe's AD), WCC uneven, B1G/SEC~0 (pooled), ACC transitioning</t>
         </is>
       </c>
       <c r="C29" s="14" t="n">

</xml_diff>